<commit_message>
Change donut-charts-wrapper to vertical flex column direction on all screen sizes under 768px (covering tablets and mobile landscape/portrait) to prevent chart squishing and overlapping labels
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -1554,7 +1554,7 @@
       </c>
       <c r="N2" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O2" s="19" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="N3" s="23" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O3" s="23" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="N4" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O4" s="19" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="N5" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O5" s="23" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>NEW ORDER</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O6" s="19" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>IN TRANSIT-EN-ROUTE</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O12" s="19" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="N13" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT-EN-ROUTE</t>
+          <t>IN TRANSIT-AT DESTINATION HUB</t>
         </is>
       </c>
       <c r="O13" s="23" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="N15" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT-EN-ROUTE</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O15" s="23" t="inlineStr">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>IN TRANSIT-EN-ROUTE</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O18" s="19" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="N19" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O19" s="23" t="inlineStr">
@@ -2943,7 +2943,7 @@
       </c>
       <c r="K20" s="20" t="inlineStr">
         <is>
-          <t>Seller Initiated Delay</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L20" s="20" t="inlineStr">
@@ -2958,12 +2958,12 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O20" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P20" s="19" t="inlineStr">
@@ -3036,7 +3036,7 @@
       </c>
       <c r="N21" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>OUT FOR DELIVERY</t>
         </is>
       </c>
       <c r="O21" s="23" t="inlineStr">
@@ -3114,12 +3114,12 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O22" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P22" s="19" t="inlineStr">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="N23" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT-AT DESTINATION HUB</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O23" s="23" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O24" s="19" t="inlineStr">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="N27" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O27" s="23" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="N29" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT-AT DESTINATION HUB</t>
+          <t>OUT FOR DELIVERY</t>
         </is>
       </c>
       <c r="O29" s="23" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="K32" s="20" t="inlineStr">
         <is>
-          <t>Customerunavailable Deliveryattempted</t>
+          <t>Deliveryattempted Unabletocontactrecipient</t>
         </is>
       </c>
       <c r="L32" s="20" t="inlineStr">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="K34" s="20" t="inlineStr">
         <is>
-          <t>Unabletocontactrecipient Deliveryattempted</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L34" s="20" t="inlineStr">
@@ -4050,12 +4050,12 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>UNDELIVERED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O34" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P34" s="19" t="inlineStr">
@@ -4128,12 +4128,12 @@
       </c>
       <c r="N35" s="23" t="inlineStr">
         <is>
-          <t>REACHED DESTINATION HUB</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O35" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P35" s="23" t="inlineStr">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="N41" s="23" t="inlineStr">
         <is>
-          <t>RTO IN TRANSIT</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O41" s="23" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>RTO IN TRANSIT</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O64" s="19" t="inlineStr">
@@ -6468,7 +6468,7 @@
       </c>
       <c r="N65" s="23" t="inlineStr">
         <is>
-          <t>RTO IN TRANSIT</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O65" s="23" t="inlineStr">
@@ -6989,7 +6989,7 @@
       </c>
       <c r="K3" s="24" t="inlineStr">
         <is>
-          <t>Unabletocontactrecipient Deliveryattempted</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L3" s="24" t="inlineStr">
@@ -7004,12 +7004,12 @@
       </c>
       <c r="N3" s="23" t="inlineStr">
         <is>
-          <t>UNDELIVERED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O3" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P3" s="23" t="inlineStr">
@@ -7082,12 +7082,12 @@
       </c>
       <c r="N4" s="19" t="inlineStr">
         <is>
-          <t>REACHED DESTINATION HUB</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O4" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P4" s="19" t="inlineStr">
@@ -7550,7 +7550,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>RTO IN TRANSIT</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O10" s="19" t="inlineStr">
@@ -9344,7 +9344,7 @@
       </c>
       <c r="N33" s="23" t="inlineStr">
         <is>
-          <t>RTO IN TRANSIT</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O33" s="23" t="inlineStr">
@@ -9422,7 +9422,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>RTO IN TRANSIT</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O34" s="19" t="inlineStr">
@@ -9726,7 +9726,7 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="41" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="33" customWidth="1" min="14" max="14"/>
@@ -9880,7 +9880,7 @@
       </c>
       <c r="N2" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O2" s="19" t="inlineStr">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="N3" s="23" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O3" s="23" t="inlineStr">
@@ -10036,7 +10036,7 @@
       </c>
       <c r="N4" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O4" s="19" t="inlineStr">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="N5" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O5" s="23" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>NEW ORDER</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O6" s="19" t="inlineStr">
@@ -10660,7 +10660,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>IN TRANSIT-EN-ROUTE</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O12" s="19" t="inlineStr">
@@ -10738,7 +10738,7 @@
       </c>
       <c r="N13" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT-EN-ROUTE</t>
+          <t>IN TRANSIT-AT DESTINATION HUB</t>
         </is>
       </c>
       <c r="O13" s="23" t="inlineStr">
@@ -10894,7 +10894,7 @@
       </c>
       <c r="N15" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT-EN-ROUTE</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O15" s="23" t="inlineStr">
@@ -11128,7 +11128,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>IN TRANSIT-EN-ROUTE</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O18" s="19" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="N19" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O19" s="23" t="inlineStr">
@@ -11269,7 +11269,7 @@
       </c>
       <c r="K20" s="20" t="inlineStr">
         <is>
-          <t>Seller Initiated Delay</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L20" s="20" t="inlineStr">
@@ -11284,12 +11284,12 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O20" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P20" s="19" t="inlineStr">
@@ -11362,7 +11362,7 @@
       </c>
       <c r="N21" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>OUT FOR DELIVERY</t>
         </is>
       </c>
       <c r="O21" s="23" t="inlineStr">
@@ -11440,12 +11440,12 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O22" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P22" s="19" t="inlineStr">
@@ -11518,7 +11518,7 @@
       </c>
       <c r="N23" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT-AT DESTINATION HUB</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O23" s="23" t="inlineStr">
@@ -11596,7 +11596,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O24" s="19" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="N27" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O27" s="23" t="inlineStr">
@@ -11986,7 +11986,7 @@
       </c>
       <c r="N29" s="23" t="inlineStr">
         <is>
-          <t>IN TRANSIT-AT DESTINATION HUB</t>
+          <t>OUT FOR DELIVERY</t>
         </is>
       </c>
       <c r="O29" s="23" t="inlineStr">
@@ -12205,7 +12205,7 @@
       </c>
       <c r="K32" s="20" t="inlineStr">
         <is>
-          <t>Customerunavailable Deliveryattempted</t>
+          <t>Deliveryattempted Unabletocontactrecipient</t>
         </is>
       </c>
       <c r="L32" s="20" t="inlineStr">

</xml_diff>

<commit_message>
Implement Shiprocket tracking: AWB Code column, Tracking Link column, interactive links in table, and details modal button
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -1045,7 +1045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1064,6 +1064,8 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1145,6 +1147,16 @@
       <c r="P1" s="10" t="inlineStr">
         <is>
           <t>Feedback Received (Yes/No)</t>
+        </is>
+      </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1178,6 +1190,8 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1259,6 +1273,16 @@
       <c r="P1" s="10" t="inlineStr">
         <is>
           <t>Feedback Received (Yes/No)</t>
+        </is>
+      </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1292,6 +1316,8 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1373,6 +1399,16 @@
       <c r="P1" s="10" t="inlineStr">
         <is>
           <t>Feedback Received (Yes/No)</t>
+        </is>
+      </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P69"/>
+  <dimension ref="A1:R69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1406,6 +1442,8 @@
     <col width="33" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1489,6 +1527,16 @@
           <t>Feedback Received (Yes/No)</t>
         </is>
       </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
@@ -1567,6 +1615,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q2" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R2" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="23" t="inlineStr">
@@ -1645,6 +1703,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q3" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R3" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -1723,6 +1791,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q4" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R4" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="23" t="inlineStr">
@@ -1801,6 +1879,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q5" s="23" t="inlineStr">
+        <is>
+          <t>SF3158681570SPF</t>
+        </is>
+      </c>
+      <c r="R5" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3158681570SPF</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
@@ -1879,6 +1967,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q6" s="19" t="inlineStr">
+        <is>
+          <t>19041933834995</t>
+        </is>
+      </c>
+      <c r="R6" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041933834995</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="23" t="inlineStr">
@@ -1957,6 +2055,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q7" s="23" t="inlineStr">
+        <is>
+          <t>19041933767110</t>
+        </is>
+      </c>
+      <c r="R7" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041933767110</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -2035,6 +2143,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q8" s="19" t="inlineStr">
+        <is>
+          <t>SF3158681535SPF</t>
+        </is>
+      </c>
+      <c r="R8" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3158681535SPF</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="23" t="inlineStr">
@@ -2113,6 +2231,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q9" s="23" t="inlineStr">
+        <is>
+          <t>7D125041276</t>
+        </is>
+      </c>
+      <c r="R9" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D125041276</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -2191,6 +2319,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q10" s="19" t="inlineStr">
+        <is>
+          <t>143263608413636</t>
+        </is>
+      </c>
+      <c r="R10" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/143263608413636</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="23" t="inlineStr">
@@ -2269,6 +2407,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q11" s="23" t="inlineStr">
+        <is>
+          <t>SF3622719795KR</t>
+        </is>
+      </c>
+      <c r="R11" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3622719795KR</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
@@ -2347,6 +2495,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q12" s="19" t="inlineStr">
+        <is>
+          <t>19041933357982</t>
+        </is>
+      </c>
+      <c r="R12" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041933357982</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="23" t="inlineStr">
@@ -2425,6 +2583,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q13" s="23" t="inlineStr">
+        <is>
+          <t>19041933358111</t>
+        </is>
+      </c>
+      <c r="R13" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041933358111</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
@@ -2503,6 +2671,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q14" s="19" t="inlineStr">
+        <is>
+          <t>19041933375224</t>
+        </is>
+      </c>
+      <c r="R14" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041933375224</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="23" t="inlineStr">
@@ -2581,6 +2759,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q15" s="23" t="inlineStr">
+        <is>
+          <t>143263612093343</t>
+        </is>
+      </c>
+      <c r="R15" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/143263612093343</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
@@ -2659,6 +2847,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q16" s="19" t="inlineStr">
+        <is>
+          <t>370577344761</t>
+        </is>
+      </c>
+      <c r="R16" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370577344761</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="23" t="inlineStr">
@@ -2737,6 +2935,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q17" s="23" t="inlineStr">
+        <is>
+          <t>14112362996290</t>
+        </is>
+      </c>
+      <c r="R17" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112362996290</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="19" t="inlineStr">
@@ -2815,6 +3023,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q18" s="19" t="inlineStr">
+        <is>
+          <t>143263608436527</t>
+        </is>
+      </c>
+      <c r="R18" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/143263608436527</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="23" t="inlineStr">
@@ -2893,6 +3111,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q19" s="23" t="inlineStr">
+        <is>
+          <t>370574614355</t>
+        </is>
+      </c>
+      <c r="R19" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370574614355</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
@@ -2971,6 +3199,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q20" s="19" t="inlineStr">
+        <is>
+          <t>SF3158680701SPF</t>
+        </is>
+      </c>
+      <c r="R20" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3158680701SPF</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="23" t="inlineStr">
@@ -3049,6 +3287,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q21" s="23" t="inlineStr">
+        <is>
+          <t>370554649599</t>
+        </is>
+      </c>
+      <c r="R21" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370554649599</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
@@ -3127,6 +3375,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q22" s="19" t="inlineStr">
+        <is>
+          <t>370552365989</t>
+        </is>
+      </c>
+      <c r="R22" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370552365989</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="23" t="inlineStr">
@@ -3205,6 +3463,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q23" s="23" t="inlineStr">
+        <is>
+          <t>1091393193440</t>
+        </is>
+      </c>
+      <c r="R23" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/1091393193440</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
@@ -3283,6 +3551,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q24" s="19" t="inlineStr">
+        <is>
+          <t>SF3158680814SPF</t>
+        </is>
+      </c>
+      <c r="R24" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3158680814SPF</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="23" t="inlineStr">
@@ -3361,6 +3639,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q25" s="23" t="inlineStr">
+        <is>
+          <t>7D131505337</t>
+        </is>
+      </c>
+      <c r="R25" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D131505337</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="19" t="inlineStr">
@@ -3439,6 +3727,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q26" s="19" t="inlineStr">
+        <is>
+          <t>370553698802</t>
+        </is>
+      </c>
+      <c r="R26" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370553698802</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="23" t="inlineStr">
@@ -3517,6 +3815,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q27" s="23" t="inlineStr">
+        <is>
+          <t>370550963576</t>
+        </is>
+      </c>
+      <c r="R27" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370550963576</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="19" t="inlineStr">
@@ -3595,6 +3903,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q28" s="19" t="inlineStr">
+        <is>
+          <t>14112362403829</t>
+        </is>
+      </c>
+      <c r="R28" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112362403829</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="23" t="inlineStr">
@@ -3673,6 +3991,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q29" s="23" t="inlineStr">
+        <is>
+          <t>1091393138630</t>
+        </is>
+      </c>
+      <c r="R29" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/1091393138630</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="19" t="inlineStr">
@@ -3751,6 +4079,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q30" s="19" t="inlineStr">
+        <is>
+          <t>7D131502192</t>
+        </is>
+      </c>
+      <c r="R30" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D131502192</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="23" t="inlineStr">
@@ -3829,6 +4167,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q31" s="23" t="inlineStr">
+        <is>
+          <t>7D131501705</t>
+        </is>
+      </c>
+      <c r="R31" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D131501705</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="19" t="inlineStr">
@@ -3907,6 +4255,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q32" s="19" t="inlineStr">
+        <is>
+          <t>370526573181</t>
+        </is>
+      </c>
+      <c r="R32" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370526573181</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="23" t="inlineStr">
@@ -3985,6 +4343,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q33" s="23" t="inlineStr">
+        <is>
+          <t>14112365216334</t>
+        </is>
+      </c>
+      <c r="R33" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112365216334</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="19" t="inlineStr">
@@ -4063,6 +4431,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q34" s="19" t="inlineStr">
+        <is>
+          <t>370503334064</t>
+        </is>
+      </c>
+      <c r="R34" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370503334064</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="23" t="inlineStr">
@@ -4141,6 +4519,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q35" s="23" t="inlineStr">
+        <is>
+          <t>370503560906</t>
+        </is>
+      </c>
+      <c r="R35" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370503560906</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="19" t="inlineStr">
@@ -4219,6 +4607,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q36" s="19" t="inlineStr">
+        <is>
+          <t>19041932647740</t>
+        </is>
+      </c>
+      <c r="R36" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041932647740</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="23" t="inlineStr">
@@ -4297,6 +4695,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q37" s="23" t="inlineStr">
+        <is>
+          <t>370494726459</t>
+        </is>
+      </c>
+      <c r="R37" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370494726459</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="19" t="inlineStr">
@@ -4375,6 +4783,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q38" s="19" t="inlineStr">
+        <is>
+          <t>7D131169474</t>
+        </is>
+      </c>
+      <c r="R38" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D131169474</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="23" t="inlineStr">
@@ -4453,6 +4871,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q39" s="23" t="inlineStr">
+        <is>
+          <t>SRSC0319007800</t>
+        </is>
+      </c>
+      <c r="R39" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSC0319007800</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="19" t="inlineStr">
@@ -4531,6 +4959,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q40" s="19" t="inlineStr">
+        <is>
+          <t>SF3593208175KR</t>
+        </is>
+      </c>
+      <c r="R40" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3593208175KR</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="23" t="inlineStr">
@@ -4609,6 +5047,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q41" s="23" t="inlineStr">
+        <is>
+          <t>14112364415189</t>
+        </is>
+      </c>
+      <c r="R41" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112364415189</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="19" t="inlineStr">
@@ -4687,6 +5135,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q42" s="19" t="inlineStr">
+        <is>
+          <t>SRSC9436482183</t>
+        </is>
+      </c>
+      <c r="R42" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSC9436482183</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="23" t="inlineStr">
@@ -4765,6 +5223,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q43" s="23" t="inlineStr">
+        <is>
+          <t>SF3158678399SPF</t>
+        </is>
+      </c>
+      <c r="R43" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3158678399SPF</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="19" t="inlineStr">
@@ -4843,6 +5311,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q44" s="19" t="inlineStr">
+        <is>
+          <t>14112363521699</t>
+        </is>
+      </c>
+      <c r="R44" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112363521699</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="23" t="inlineStr">
@@ -4921,6 +5399,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q45" s="23" t="inlineStr">
+        <is>
+          <t>14112364314371</t>
+        </is>
+      </c>
+      <c r="R45" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112364314371</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="19" t="inlineStr">
@@ -4999,6 +5487,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q46" s="19" t="inlineStr">
+        <is>
+          <t>14112363687734</t>
+        </is>
+      </c>
+      <c r="R46" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112363687734</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="23" t="inlineStr">
@@ -5077,6 +5575,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q47" s="23" t="inlineStr">
+        <is>
+          <t>370430051263</t>
+        </is>
+      </c>
+      <c r="R47" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370430051263</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="19" t="inlineStr">
@@ -5155,6 +5663,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q48" s="19" t="inlineStr">
+        <is>
+          <t>14112367080297</t>
+        </is>
+      </c>
+      <c r="R48" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112367080297</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="23" t="inlineStr">
@@ -5233,6 +5751,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q49" s="23" t="inlineStr">
+        <is>
+          <t>370429882984</t>
+        </is>
+      </c>
+      <c r="R49" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370429882984</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="19" t="inlineStr">
@@ -5311,6 +5839,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q50" s="19" t="inlineStr">
+        <is>
+          <t>14112365054938</t>
+        </is>
+      </c>
+      <c r="R50" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112365054938</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="23" t="inlineStr">
@@ -5389,6 +5927,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q51" s="23" t="inlineStr">
+        <is>
+          <t>SF3586915332KR</t>
+        </is>
+      </c>
+      <c r="R51" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3586915332KR</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="19" t="inlineStr">
@@ -5467,6 +6015,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q52" s="19" t="inlineStr">
+        <is>
+          <t>14112362848987</t>
+        </is>
+      </c>
+      <c r="R52" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112362848987</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="23" t="inlineStr">
@@ -5545,6 +6103,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q53" s="23" t="inlineStr">
+        <is>
+          <t>370429573110</t>
+        </is>
+      </c>
+      <c r="R53" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370429573110</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="19" t="inlineStr">
@@ -5623,6 +6191,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q54" s="19" t="inlineStr">
+        <is>
+          <t>14112363585911</t>
+        </is>
+      </c>
+      <c r="R54" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112363585911</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="23" t="inlineStr">
@@ -5701,6 +6279,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q55" s="23" t="inlineStr">
+        <is>
+          <t>7D131457369</t>
+        </is>
+      </c>
+      <c r="R55" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D131457369</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="19" t="inlineStr">
@@ -5779,6 +6367,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q56" s="19" t="inlineStr">
+        <is>
+          <t>370395354997</t>
+        </is>
+      </c>
+      <c r="R56" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370395354997</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="23" t="inlineStr">
@@ -5857,6 +6455,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="Q57" s="23" t="inlineStr">
+        <is>
+          <t>SRSC9946388102</t>
+        </is>
+      </c>
+      <c r="R57" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSC9946388102</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="19" t="inlineStr">
@@ -5935,6 +6543,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q58" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R58" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="23" t="inlineStr">
@@ -6013,6 +6631,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q59" s="23" t="inlineStr">
+        <is>
+          <t>SF3576445793KR</t>
+        </is>
+      </c>
+      <c r="R59" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3576445793KR</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="19" t="inlineStr">
@@ -6091,6 +6719,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q60" s="19" t="inlineStr">
+        <is>
+          <t>SRSC3884345902</t>
+        </is>
+      </c>
+      <c r="R60" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSC3884345902</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="23" t="inlineStr">
@@ -6169,6 +6807,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q61" s="23" t="inlineStr">
+        <is>
+          <t>370384504495</t>
+        </is>
+      </c>
+      <c r="R61" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370384504495</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="19" t="inlineStr">
@@ -6247,6 +6895,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q62" s="19" t="inlineStr">
+        <is>
+          <t>SRSP2020476035</t>
+        </is>
+      </c>
+      <c r="R62" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSP2020476035</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="23" t="inlineStr">
@@ -6325,6 +6983,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q63" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R63" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="19" t="inlineStr">
@@ -6403,6 +7071,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q64" s="19" t="inlineStr">
+        <is>
+          <t>1319460341769</t>
+        </is>
+      </c>
+      <c r="R64" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/1319460341769</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="A65" s="23" t="inlineStr">
@@ -6481,6 +7159,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q65" s="23" t="inlineStr">
+        <is>
+          <t>1319460341773</t>
+        </is>
+      </c>
+      <c r="R65" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/1319460341773</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="A66" s="19" t="inlineStr">
@@ -6559,6 +7247,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q66" s="19" t="inlineStr">
+        <is>
+          <t>14112362553816</t>
+        </is>
+      </c>
+      <c r="R66" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112362553816</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="23" t="inlineStr">
@@ -6637,6 +7335,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q67" s="23" t="inlineStr">
+        <is>
+          <t>SRSP8409363746</t>
+        </is>
+      </c>
+      <c r="R67" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSP8409363746</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="19" t="inlineStr">
@@ -6713,6 +7421,16 @@
       <c r="P68" s="19" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="Q68" s="19" t="inlineStr">
+        <is>
+          <t>14112363889759</t>
+        </is>
+      </c>
+      <c r="R68" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112363889759</t>
         </is>
       </c>
     </row>
@@ -6747,6 +7465,8 @@
       <c r="N69" s="27" t="n"/>
       <c r="O69" s="27" t="n"/>
       <c r="P69" s="27" t="n"/>
+      <c r="Q69" s="27" t="n"/>
+      <c r="R69" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6759,7 +7479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:R38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6778,6 +7498,8 @@
     <col width="27" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -6861,6 +7583,16 @@
           <t>Feedback Received (Yes/No)</t>
         </is>
       </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
@@ -6939,6 +7671,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q2" s="19" t="inlineStr">
+        <is>
+          <t>14112365216334</t>
+        </is>
+      </c>
+      <c r="R2" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112365216334</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="23" t="inlineStr">
@@ -7017,6 +7759,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q3" s="23" t="inlineStr">
+        <is>
+          <t>370503334064</t>
+        </is>
+      </c>
+      <c r="R3" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370503334064</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -7095,6 +7847,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q4" s="19" t="inlineStr">
+        <is>
+          <t>370503560906</t>
+        </is>
+      </c>
+      <c r="R4" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370503560906</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="23" t="inlineStr">
@@ -7173,6 +7935,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q5" s="23" t="inlineStr">
+        <is>
+          <t>19041932647740</t>
+        </is>
+      </c>
+      <c r="R5" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041932647740</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
@@ -7251,6 +8023,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q6" s="19" t="inlineStr">
+        <is>
+          <t>370494726459</t>
+        </is>
+      </c>
+      <c r="R6" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370494726459</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="23" t="inlineStr">
@@ -7329,6 +8111,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q7" s="23" t="inlineStr">
+        <is>
+          <t>7D131169474</t>
+        </is>
+      </c>
+      <c r="R7" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D131169474</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -7407,6 +8199,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q8" s="19" t="inlineStr">
+        <is>
+          <t>SRSC0319007800</t>
+        </is>
+      </c>
+      <c r="R8" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSC0319007800</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="23" t="inlineStr">
@@ -7485,6 +8287,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q9" s="23" t="inlineStr">
+        <is>
+          <t>SF3593208175KR</t>
+        </is>
+      </c>
+      <c r="R9" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3593208175KR</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -7563,6 +8375,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q10" s="19" t="inlineStr">
+        <is>
+          <t>14112364415189</t>
+        </is>
+      </c>
+      <c r="R10" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112364415189</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="23" t="inlineStr">
@@ -7641,6 +8463,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q11" s="23" t="inlineStr">
+        <is>
+          <t>SRSC9436482183</t>
+        </is>
+      </c>
+      <c r="R11" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSC9436482183</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
@@ -7719,6 +8551,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q12" s="19" t="inlineStr">
+        <is>
+          <t>SF3158678399SPF</t>
+        </is>
+      </c>
+      <c r="R12" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3158678399SPF</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="23" t="inlineStr">
@@ -7797,6 +8639,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q13" s="23" t="inlineStr">
+        <is>
+          <t>14112363521699</t>
+        </is>
+      </c>
+      <c r="R13" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112363521699</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
@@ -7875,6 +8727,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q14" s="19" t="inlineStr">
+        <is>
+          <t>14112364314371</t>
+        </is>
+      </c>
+      <c r="R14" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112364314371</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="23" t="inlineStr">
@@ -7953,6 +8815,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q15" s="23" t="inlineStr">
+        <is>
+          <t>14112363687734</t>
+        </is>
+      </c>
+      <c r="R15" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112363687734</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
@@ -8031,6 +8903,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q16" s="19" t="inlineStr">
+        <is>
+          <t>370430051263</t>
+        </is>
+      </c>
+      <c r="R16" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370430051263</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="23" t="inlineStr">
@@ -8109,6 +8991,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q17" s="23" t="inlineStr">
+        <is>
+          <t>14112367080297</t>
+        </is>
+      </c>
+      <c r="R17" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112367080297</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="19" t="inlineStr">
@@ -8187,6 +9079,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q18" s="19" t="inlineStr">
+        <is>
+          <t>370429882984</t>
+        </is>
+      </c>
+      <c r="R18" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370429882984</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="23" t="inlineStr">
@@ -8265,6 +9167,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q19" s="23" t="inlineStr">
+        <is>
+          <t>14112365054938</t>
+        </is>
+      </c>
+      <c r="R19" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112365054938</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
@@ -8343,6 +9255,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q20" s="19" t="inlineStr">
+        <is>
+          <t>SF3586915332KR</t>
+        </is>
+      </c>
+      <c r="R20" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3586915332KR</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="23" t="inlineStr">
@@ -8421,6 +9343,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q21" s="23" t="inlineStr">
+        <is>
+          <t>14112362848987</t>
+        </is>
+      </c>
+      <c r="R21" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112362848987</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
@@ -8499,6 +9431,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q22" s="19" t="inlineStr">
+        <is>
+          <t>370429573110</t>
+        </is>
+      </c>
+      <c r="R22" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370429573110</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="23" t="inlineStr">
@@ -8577,6 +9519,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q23" s="23" t="inlineStr">
+        <is>
+          <t>14112363585911</t>
+        </is>
+      </c>
+      <c r="R23" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112363585911</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
@@ -8655,6 +9607,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q24" s="19" t="inlineStr">
+        <is>
+          <t>7D131457369</t>
+        </is>
+      </c>
+      <c r="R24" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D131457369</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="23" t="inlineStr">
@@ -8733,6 +9695,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q25" s="23" t="inlineStr">
+        <is>
+          <t>370395354997</t>
+        </is>
+      </c>
+      <c r="R25" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370395354997</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="19" t="inlineStr">
@@ -8811,6 +9783,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="Q26" s="19" t="inlineStr">
+        <is>
+          <t>SRSC9946388102</t>
+        </is>
+      </c>
+      <c r="R26" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSC9946388102</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="23" t="inlineStr">
@@ -8889,6 +9871,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q27" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R27" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="19" t="inlineStr">
@@ -8967,6 +9959,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q28" s="19" t="inlineStr">
+        <is>
+          <t>SF3576445793KR</t>
+        </is>
+      </c>
+      <c r="R28" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3576445793KR</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="23" t="inlineStr">
@@ -9045,6 +10047,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q29" s="23" t="inlineStr">
+        <is>
+          <t>SRSC3884345902</t>
+        </is>
+      </c>
+      <c r="R29" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSC3884345902</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="19" t="inlineStr">
@@ -9123,6 +10135,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q30" s="19" t="inlineStr">
+        <is>
+          <t>370384504495</t>
+        </is>
+      </c>
+      <c r="R30" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370384504495</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="23" t="inlineStr">
@@ -9201,6 +10223,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q31" s="23" t="inlineStr">
+        <is>
+          <t>SRSP2020476035</t>
+        </is>
+      </c>
+      <c r="R31" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSP2020476035</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="19" t="inlineStr">
@@ -9279,6 +10311,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q32" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R32" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="23" t="inlineStr">
@@ -9357,6 +10399,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q33" s="23" t="inlineStr">
+        <is>
+          <t>1319460341769</t>
+        </is>
+      </c>
+      <c r="R33" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/1319460341769</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="19" t="inlineStr">
@@ -9435,6 +10487,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q34" s="19" t="inlineStr">
+        <is>
+          <t>1319460341773</t>
+        </is>
+      </c>
+      <c r="R34" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/1319460341773</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="23" t="inlineStr">
@@ -9513,6 +10575,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q35" s="23" t="inlineStr">
+        <is>
+          <t>14112362553816</t>
+        </is>
+      </c>
+      <c r="R35" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112362553816</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="19" t="inlineStr">
@@ -9591,6 +10663,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q36" s="19" t="inlineStr">
+        <is>
+          <t>SRSP8409363746</t>
+        </is>
+      </c>
+      <c r="R36" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SRSP8409363746</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="23" t="inlineStr">
@@ -9667,6 +10749,16 @@
       <c r="P37" s="23" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="Q37" s="23" t="inlineStr">
+        <is>
+          <t>14112363889759</t>
+        </is>
+      </c>
+      <c r="R37" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112363889759</t>
         </is>
       </c>
     </row>
@@ -9701,6 +10793,8 @@
       <c r="N38" s="27" t="n"/>
       <c r="O38" s="27" t="n"/>
       <c r="P38" s="27" t="n"/>
+      <c r="Q38" s="27" t="n"/>
+      <c r="R38" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9713,7 +10807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9732,6 +10826,8 @@
     <col width="33" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -9815,6 +10911,16 @@
           <t>Feedback Received (Yes/No)</t>
         </is>
       </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
@@ -9893,6 +10999,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q2" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R2" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="23" t="inlineStr">
@@ -9971,6 +11087,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q3" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R3" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -10049,6 +11175,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q4" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R4" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="23" t="inlineStr">
@@ -10127,6 +11263,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q5" s="23" t="inlineStr">
+        <is>
+          <t>SF3158681570SPF</t>
+        </is>
+      </c>
+      <c r="R5" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3158681570SPF</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
@@ -10205,6 +11351,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q6" s="19" t="inlineStr">
+        <is>
+          <t>19041933834995</t>
+        </is>
+      </c>
+      <c r="R6" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041933834995</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="23" t="inlineStr">
@@ -10283,6 +11439,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q7" s="23" t="inlineStr">
+        <is>
+          <t>19041933767110</t>
+        </is>
+      </c>
+      <c r="R7" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041933767110</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -10361,6 +11527,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q8" s="19" t="inlineStr">
+        <is>
+          <t>SF3158681535SPF</t>
+        </is>
+      </c>
+      <c r="R8" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3158681535SPF</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="23" t="inlineStr">
@@ -10439,6 +11615,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q9" s="23" t="inlineStr">
+        <is>
+          <t>7D125041276</t>
+        </is>
+      </c>
+      <c r="R9" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D125041276</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -10517,6 +11703,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q10" s="19" t="inlineStr">
+        <is>
+          <t>143263608413636</t>
+        </is>
+      </c>
+      <c r="R10" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/143263608413636</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="23" t="inlineStr">
@@ -10595,6 +11791,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q11" s="23" t="inlineStr">
+        <is>
+          <t>SF3622719795KR</t>
+        </is>
+      </c>
+      <c r="R11" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3622719795KR</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
@@ -10673,6 +11879,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q12" s="19" t="inlineStr">
+        <is>
+          <t>19041933357982</t>
+        </is>
+      </c>
+      <c r="R12" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041933357982</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="23" t="inlineStr">
@@ -10751,6 +11967,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q13" s="23" t="inlineStr">
+        <is>
+          <t>19041933358111</t>
+        </is>
+      </c>
+      <c r="R13" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041933358111</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
@@ -10829,6 +12055,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q14" s="19" t="inlineStr">
+        <is>
+          <t>19041933375224</t>
+        </is>
+      </c>
+      <c r="R14" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/19041933375224</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="23" t="inlineStr">
@@ -10907,6 +12143,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q15" s="23" t="inlineStr">
+        <is>
+          <t>143263612093343</t>
+        </is>
+      </c>
+      <c r="R15" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/143263612093343</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
@@ -10985,6 +12231,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q16" s="19" t="inlineStr">
+        <is>
+          <t>370577344761</t>
+        </is>
+      </c>
+      <c r="R16" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370577344761</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="23" t="inlineStr">
@@ -11063,6 +12319,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q17" s="23" t="inlineStr">
+        <is>
+          <t>14112362996290</t>
+        </is>
+      </c>
+      <c r="R17" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112362996290</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="19" t="inlineStr">
@@ -11141,6 +12407,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q18" s="19" t="inlineStr">
+        <is>
+          <t>143263608436527</t>
+        </is>
+      </c>
+      <c r="R18" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/143263608436527</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="23" t="inlineStr">
@@ -11219,6 +12495,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q19" s="23" t="inlineStr">
+        <is>
+          <t>370574614355</t>
+        </is>
+      </c>
+      <c r="R19" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370574614355</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
@@ -11297,6 +12583,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q20" s="19" t="inlineStr">
+        <is>
+          <t>SF3158680701SPF</t>
+        </is>
+      </c>
+      <c r="R20" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3158680701SPF</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="23" t="inlineStr">
@@ -11375,6 +12671,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q21" s="23" t="inlineStr">
+        <is>
+          <t>370554649599</t>
+        </is>
+      </c>
+      <c r="R21" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370554649599</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
@@ -11453,6 +12759,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q22" s="19" t="inlineStr">
+        <is>
+          <t>370552365989</t>
+        </is>
+      </c>
+      <c r="R22" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370552365989</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="23" t="inlineStr">
@@ -11531,6 +12847,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q23" s="23" t="inlineStr">
+        <is>
+          <t>1091393193440</t>
+        </is>
+      </c>
+      <c r="R23" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/1091393193440</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
@@ -11609,6 +12935,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q24" s="19" t="inlineStr">
+        <is>
+          <t>SF3158680814SPF</t>
+        </is>
+      </c>
+      <c r="R24" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/SF3158680814SPF</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="23" t="inlineStr">
@@ -11687,6 +13023,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q25" s="23" t="inlineStr">
+        <is>
+          <t>7D131505337</t>
+        </is>
+      </c>
+      <c r="R25" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D131505337</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="19" t="inlineStr">
@@ -11765,6 +13111,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q26" s="19" t="inlineStr">
+        <is>
+          <t>370553698802</t>
+        </is>
+      </c>
+      <c r="R26" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370553698802</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="23" t="inlineStr">
@@ -11843,6 +13199,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q27" s="23" t="inlineStr">
+        <is>
+          <t>370550963576</t>
+        </is>
+      </c>
+      <c r="R27" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370550963576</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="19" t="inlineStr">
@@ -11921,6 +13287,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q28" s="19" t="inlineStr">
+        <is>
+          <t>14112362403829</t>
+        </is>
+      </c>
+      <c r="R28" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/14112362403829</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="23" t="inlineStr">
@@ -11999,6 +13375,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q29" s="23" t="inlineStr">
+        <is>
+          <t>1091393138630</t>
+        </is>
+      </c>
+      <c r="R29" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/1091393138630</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="19" t="inlineStr">
@@ -12077,6 +13463,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q30" s="19" t="inlineStr">
+        <is>
+          <t>7D131502192</t>
+        </is>
+      </c>
+      <c r="R30" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D131502192</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="23" t="inlineStr">
@@ -12155,6 +13551,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="Q31" s="23" t="inlineStr">
+        <is>
+          <t>7D131501705</t>
+        </is>
+      </c>
+      <c r="R31" s="23" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/7D131501705</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="19" t="inlineStr">
@@ -12231,6 +13637,16 @@
       <c r="P32" s="19" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="Q32" s="19" t="inlineStr">
+        <is>
+          <t>370526573181</t>
+        </is>
+      </c>
+      <c r="R32" s="19" t="inlineStr">
+        <is>
+          <t>https://shiprocket.co/tracking/370526573181</t>
         </is>
       </c>
     </row>
@@ -12265,6 +13681,8 @@
       <c r="N33" s="27" t="n"/>
       <c r="O33" s="27" t="n"/>
       <c r="P33" s="27" t="n"/>
+      <c r="Q33" s="27" t="n"/>
+      <c r="R33" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12277,7 +13695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12296,6 +13714,8 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -12377,6 +13797,16 @@
       <c r="P1" s="10" t="inlineStr">
         <is>
           <t>Feedback Received (Yes/No)</t>
+        </is>
+      </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
         </is>
       </c>
     </row>
@@ -12391,7 +13821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12410,6 +13840,8 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -12491,6 +13923,16 @@
       <c r="P1" s="10" t="inlineStr">
         <is>
           <t>Feedback Received (Yes/No)</t>
+        </is>
+      </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
         </is>
       </c>
     </row>
@@ -12505,7 +13947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12524,6 +13966,8 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -12605,6 +14049,16 @@
       <c r="P1" s="10" t="inlineStr">
         <is>
           <t>Feedback Received (Yes/No)</t>
+        </is>
+      </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
         </is>
       </c>
     </row>
@@ -12619,7 +14073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12638,6 +14092,8 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -12719,6 +14175,16 @@
       <c r="P1" s="10" t="inlineStr">
         <is>
           <t>Feedback Received (Yes/No)</t>
+        </is>
+      </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
         </is>
       </c>
     </row>
@@ -12733,7 +14199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12752,6 +14218,8 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -12835,6 +14303,16 @@
           <t>Feedback Received (Yes/No)</t>
         </is>
       </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>AWB Code</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>Tracking Link</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Restore historical tracking details by merging Shiprocket CSV database
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -715,16 +715,16 @@
         <v>107964</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>1032</v>
+        <v>9726</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>106932</v>
+        <v>98238</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>0.01408450704225352</v>
+        <v>0.08450704225352113</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>0</v>
+        <v>0.1136363636363636</v>
       </c>
     </row>
     <row r="6">
@@ -1449,14 +1449,14 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="33" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O6" s="19" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="N7" s="23" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O7" s="23" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O8" s="19" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="N9" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O9" s="23" t="inlineStr">
@@ -2246,12 +2246,12 @@
       </c>
       <c r="Q9" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3158681570SPF</t>
         </is>
       </c>
       <c r="R9" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3158681570SPF</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O10" s="19" t="inlineStr">
@@ -2334,12 +2334,12 @@
       </c>
       <c r="Q10" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041933834995</t>
         </is>
       </c>
       <c r="R10" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041933834995</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="N11" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O11" s="23" t="inlineStr">
@@ -2422,12 +2422,12 @@
       </c>
       <c r="Q11" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041933767110</t>
         </is>
       </c>
       <c r="R11" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041933767110</t>
         </is>
       </c>
     </row>
@@ -2495,7 +2495,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O12" s="19" t="inlineStr">
@@ -2510,12 +2510,12 @@
       </c>
       <c r="Q12" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3158681535SPF</t>
         </is>
       </c>
       <c r="R12" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3158681535SPF</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="N13" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>OUT FOR PICKUP</t>
         </is>
       </c>
       <c r="O13" s="23" t="inlineStr">
@@ -2598,12 +2598,12 @@
       </c>
       <c r="Q13" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D125041276</t>
         </is>
       </c>
       <c r="R13" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D125041276</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>IN TRANSIT-EN-ROUTE</t>
         </is>
       </c>
       <c r="O14" s="19" t="inlineStr">
@@ -2686,12 +2686,12 @@
       </c>
       <c r="Q14" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>143263608413636</t>
         </is>
       </c>
       <c r="R14" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/143263608413636</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2759,7 @@
       </c>
       <c r="N15" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O15" s="23" t="inlineStr">
@@ -2774,12 +2774,12 @@
       </c>
       <c r="Q15" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3622719795KR</t>
         </is>
       </c>
       <c r="R15" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3622719795KR</t>
         </is>
       </c>
     </row>
@@ -2847,7 +2847,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O16" s="19" t="inlineStr">
@@ -2862,12 +2862,12 @@
       </c>
       <c r="Q16" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041933357982</t>
         </is>
       </c>
       <c r="R16" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041933357982</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="N17" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>IN TRANSIT-AT DESTINATION HUB</t>
         </is>
       </c>
       <c r="O17" s="23" t="inlineStr">
@@ -2950,12 +2950,12 @@
       </c>
       <c r="Q17" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041933358111</t>
         </is>
       </c>
       <c r="R17" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041933358111</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>IN TRANSIT-EN-ROUTE</t>
         </is>
       </c>
       <c r="O18" s="19" t="inlineStr">
@@ -3038,12 +3038,12 @@
       </c>
       <c r="Q18" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041933375224</t>
         </is>
       </c>
       <c r="R18" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041933375224</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="N19" s="23" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O19" s="23" t="inlineStr">
@@ -3126,12 +3126,12 @@
       </c>
       <c r="Q19" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>143263612093343</t>
         </is>
       </c>
       <c r="R19" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/143263612093343</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3199,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>IN TRANSIT</t>
         </is>
       </c>
       <c r="O20" s="19" t="inlineStr">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="Q20" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370577344761</t>
         </is>
       </c>
       <c r="R20" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370577344761</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="N21" s="23" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>IN TRANSIT-EN-ROUTE</t>
         </is>
       </c>
       <c r="O21" s="23" t="inlineStr">
@@ -3302,12 +3302,12 @@
       </c>
       <c r="Q21" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112362996290</t>
         </is>
       </c>
       <c r="R21" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112362996290</t>
         </is>
       </c>
     </row>
@@ -3375,7 +3375,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O22" s="19" t="inlineStr">
@@ -3390,12 +3390,12 @@
       </c>
       <c r="Q22" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>143263608436527</t>
         </is>
       </c>
       <c r="R22" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/143263608436527</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="N23" s="23" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O23" s="23" t="inlineStr">
@@ -3478,12 +3478,12 @@
       </c>
       <c r="Q23" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370574614355</t>
         </is>
       </c>
       <c r="R23" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370574614355</t>
         </is>
       </c>
     </row>
@@ -3551,12 +3551,12 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O24" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P24" s="19" t="inlineStr">
@@ -3566,12 +3566,12 @@
       </c>
       <c r="Q24" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3158680701SPF</t>
         </is>
       </c>
       <c r="R24" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3158680701SPF</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="N25" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>OUT FOR DELIVERY</t>
         </is>
       </c>
       <c r="O25" s="23" t="inlineStr">
@@ -3654,12 +3654,12 @@
       </c>
       <c r="Q25" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370554649599</t>
         </is>
       </c>
       <c r="R25" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370554649599</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O26" s="19" t="inlineStr">
@@ -3742,12 +3742,12 @@
       </c>
       <c r="Q26" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370552365989</t>
         </is>
       </c>
       <c r="R26" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370552365989</t>
         </is>
       </c>
     </row>
@@ -3800,7 +3800,7 @@
       </c>
       <c r="K27" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pickup Not Attempted</t>
         </is>
       </c>
       <c r="L27" s="24" t="inlineStr">
@@ -3815,7 +3815,7 @@
       </c>
       <c r="N27" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O27" s="23" t="inlineStr">
@@ -3830,12 +3830,12 @@
       </c>
       <c r="Q27" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1091393193440</t>
         </is>
       </c>
       <c r="R27" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/1091393193440</t>
         </is>
       </c>
     </row>
@@ -3903,7 +3903,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O28" s="19" t="inlineStr">
@@ -3918,12 +3918,12 @@
       </c>
       <c r="Q28" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3158680814SPF</t>
         </is>
       </c>
       <c r="R28" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3158680814SPF</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="N29" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP EXCEPTION</t>
         </is>
       </c>
       <c r="O29" s="23" t="inlineStr">
@@ -4006,12 +4006,12 @@
       </c>
       <c r="Q29" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131505337</t>
         </is>
       </c>
       <c r="R29" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131505337</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>IN TRANSIT</t>
         </is>
       </c>
       <c r="O30" s="19" t="inlineStr">
@@ -4094,12 +4094,12 @@
       </c>
       <c r="Q30" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370553698802</t>
         </is>
       </c>
       <c r="R30" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370553698802</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="N31" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O31" s="23" t="inlineStr">
@@ -4182,12 +4182,12 @@
       </c>
       <c r="Q31" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370550963576</t>
         </is>
       </c>
       <c r="R31" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370550963576</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>CANCELED</t>
         </is>
       </c>
       <c r="O32" s="19" t="inlineStr">
@@ -4270,12 +4270,12 @@
       </c>
       <c r="Q32" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112362403829</t>
         </is>
       </c>
       <c r="R32" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112362403829</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="K33" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pickup Not Attempted</t>
         </is>
       </c>
       <c r="L33" s="24" t="inlineStr">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="N33" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>OUT FOR DELIVERY</t>
         </is>
       </c>
       <c r="O33" s="23" t="inlineStr">
@@ -4358,12 +4358,12 @@
       </c>
       <c r="Q33" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1091393138630</t>
         </is>
       </c>
       <c r="R33" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/1091393138630</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP EXCEPTION</t>
         </is>
       </c>
       <c r="O34" s="19" t="inlineStr">
@@ -4446,12 +4446,12 @@
       </c>
       <c r="Q34" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131502192</t>
         </is>
       </c>
       <c r="R34" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131502192</t>
         </is>
       </c>
     </row>
@@ -4519,7 +4519,7 @@
       </c>
       <c r="N35" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP EXCEPTION</t>
         </is>
       </c>
       <c r="O35" s="23" t="inlineStr">
@@ -4534,12 +4534,12 @@
       </c>
       <c r="Q35" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131501705</t>
         </is>
       </c>
       <c r="R35" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131501705</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="K36" s="20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Deliveryattempted Unabletocontactrecipient</t>
         </is>
       </c>
       <c r="L36" s="20" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>UNDELIVERED</t>
         </is>
       </c>
       <c r="O36" s="19" t="inlineStr">
@@ -4622,12 +4622,12 @@
       </c>
       <c r="Q36" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370526573181</t>
         </is>
       </c>
       <c r="R36" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370526573181</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="N37" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O37" s="23" t="inlineStr">
@@ -4710,12 +4710,12 @@
       </c>
       <c r="Q37" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112365216334</t>
         </is>
       </c>
       <c r="R37" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112365216334</t>
         </is>
       </c>
     </row>
@@ -4783,12 +4783,12 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O38" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P38" s="19" t="inlineStr">
@@ -4798,12 +4798,12 @@
       </c>
       <c r="Q38" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370503334064</t>
         </is>
       </c>
       <c r="R38" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370503334064</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="N39" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O39" s="23" t="inlineStr">
@@ -4886,12 +4886,12 @@
       </c>
       <c r="Q39" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370503560906</t>
         </is>
       </c>
       <c r="R39" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370503560906</t>
         </is>
       </c>
     </row>
@@ -4959,12 +4959,12 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O40" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P40" s="19" t="inlineStr">
@@ -4974,12 +4974,12 @@
       </c>
       <c r="Q40" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041932647740</t>
         </is>
       </c>
       <c r="R40" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041932647740</t>
         </is>
       </c>
     </row>
@@ -5047,12 +5047,12 @@
       </c>
       <c r="N41" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O41" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P41" s="23" t="inlineStr">
@@ -5062,12 +5062,12 @@
       </c>
       <c r="Q41" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370494726459</t>
         </is>
       </c>
       <c r="R41" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370494726459</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O42" s="19" t="inlineStr">
@@ -5150,12 +5150,12 @@
       </c>
       <c r="Q42" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131169474</t>
         </is>
       </c>
       <c r="R42" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131169474</t>
         </is>
       </c>
     </row>
@@ -5223,7 +5223,7 @@
       </c>
       <c r="N43" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>UNDELIVERED-1ST ATTEMPT</t>
         </is>
       </c>
       <c r="O43" s="23" t="inlineStr">
@@ -5238,12 +5238,12 @@
       </c>
       <c r="Q43" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSC0319007800</t>
         </is>
       </c>
       <c r="R43" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSC0319007800</t>
         </is>
       </c>
     </row>
@@ -5286,17 +5286,17 @@
       </c>
       <c r="I44" s="19" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J44" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K44" s="20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Cancelled Otp Verified</t>
         </is>
       </c>
       <c r="L44" s="20" t="inlineStr">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO IN TRANSIT</t>
         </is>
       </c>
       <c r="O44" s="19" t="inlineStr">
@@ -5326,12 +5326,12 @@
       </c>
       <c r="Q44" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3593208175KR</t>
         </is>
       </c>
       <c r="R44" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3593208175KR</t>
         </is>
       </c>
     </row>
@@ -5374,17 +5374,17 @@
       </c>
       <c r="I45" s="23" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J45" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K45" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Refused To Accept   Otp Verified</t>
         </is>
       </c>
       <c r="L45" s="24" t="inlineStr">
@@ -5399,7 +5399,7 @@
       </c>
       <c r="N45" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O45" s="23" t="inlineStr">
@@ -5414,12 +5414,12 @@
       </c>
       <c r="Q45" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112364415189</t>
         </is>
       </c>
       <c r="R45" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112364415189</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O46" s="19" t="inlineStr">
@@ -5502,12 +5502,12 @@
       </c>
       <c r="Q46" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSC9436482183</t>
         </is>
       </c>
       <c r="R46" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSC9436482183</t>
         </is>
       </c>
     </row>
@@ -5575,7 +5575,7 @@
       </c>
       <c r="N47" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O47" s="23" t="inlineStr">
@@ -5590,12 +5590,12 @@
       </c>
       <c r="Q47" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3158678399SPF</t>
         </is>
       </c>
       <c r="R47" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3158678399SPF</t>
         </is>
       </c>
     </row>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O48" s="19" t="inlineStr">
@@ -5678,12 +5678,12 @@
       </c>
       <c r="Q48" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363521699</t>
         </is>
       </c>
       <c r="R48" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363521699</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="N49" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O49" s="23" t="inlineStr">
@@ -5766,12 +5766,12 @@
       </c>
       <c r="Q49" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112364314371</t>
         </is>
       </c>
       <c r="R49" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112364314371</t>
         </is>
       </c>
     </row>
@@ -5839,7 +5839,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O50" s="19" t="inlineStr">
@@ -5854,12 +5854,12 @@
       </c>
       <c r="Q50" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363687734</t>
         </is>
       </c>
       <c r="R50" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363687734</t>
         </is>
       </c>
     </row>
@@ -5927,7 +5927,7 @@
       </c>
       <c r="N51" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O51" s="23" t="inlineStr">
@@ -5942,12 +5942,12 @@
       </c>
       <c r="Q51" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370430051263</t>
         </is>
       </c>
       <c r="R51" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370430051263</t>
         </is>
       </c>
     </row>
@@ -6015,12 +6015,12 @@
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O52" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P52" s="19" t="inlineStr">
@@ -6030,12 +6030,12 @@
       </c>
       <c r="Q52" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112367080297</t>
         </is>
       </c>
       <c r="R52" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112367080297</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6103,7 @@
       </c>
       <c r="N53" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O53" s="23" t="inlineStr">
@@ -6118,12 +6118,12 @@
       </c>
       <c r="Q53" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370429882984</t>
         </is>
       </c>
       <c r="R53" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370429882984</t>
         </is>
       </c>
     </row>
@@ -6191,7 +6191,7 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O54" s="19" t="inlineStr">
@@ -6206,12 +6206,12 @@
       </c>
       <c r="Q54" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112365054938</t>
         </is>
       </c>
       <c r="R54" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112365054938</t>
         </is>
       </c>
     </row>
@@ -6279,12 +6279,12 @@
       </c>
       <c r="N55" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O55" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P55" s="23" t="inlineStr">
@@ -6294,12 +6294,12 @@
       </c>
       <c r="Q55" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3586915332KR</t>
         </is>
       </c>
       <c r="R55" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3586915332KR</t>
         </is>
       </c>
     </row>
@@ -6367,7 +6367,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O56" s="19" t="inlineStr">
@@ -6382,12 +6382,12 @@
       </c>
       <c r="Q56" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112362848987</t>
         </is>
       </c>
       <c r="R56" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112362848987</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="K57" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customerunavailable Deliveryattempted</t>
         </is>
       </c>
       <c r="L57" s="24" t="inlineStr">
@@ -6455,7 +6455,7 @@
       </c>
       <c r="N57" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>UNDELIVERED-3RD ATTEMPT</t>
         </is>
       </c>
       <c r="O57" s="23" t="inlineStr">
@@ -6470,12 +6470,12 @@
       </c>
       <c r="Q57" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370429573110</t>
         </is>
       </c>
       <c r="R57" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370429573110</t>
         </is>
       </c>
     </row>
@@ -6518,17 +6518,17 @@
       </c>
       <c r="I58" s="19" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J58" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K58" s="20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Not Available X Office Or Residence Closed</t>
         </is>
       </c>
       <c r="L58" s="20" t="inlineStr">
@@ -6543,7 +6543,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO IN TRANSIT</t>
         </is>
       </c>
       <c r="O58" s="19" t="inlineStr">
@@ -6558,12 +6558,12 @@
       </c>
       <c r="Q58" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363585911</t>
         </is>
       </c>
       <c r="R58" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363585911</t>
         </is>
       </c>
     </row>
@@ -6616,7 +6616,7 @@
       </c>
       <c r="K59" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Receiver Requested Delivery On Another Date (Cir)</t>
         </is>
       </c>
       <c r="L59" s="24" t="inlineStr">
@@ -6631,7 +6631,7 @@
       </c>
       <c r="N59" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>UNDELIVERED-1ST ATTEMPT</t>
         </is>
       </c>
       <c r="O59" s="23" t="inlineStr">
@@ -6646,12 +6646,12 @@
       </c>
       <c r="Q59" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131457369</t>
         </is>
       </c>
       <c r="R59" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131457369</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O60" s="19" t="inlineStr">
@@ -6734,12 +6734,12 @@
       </c>
       <c r="Q60" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370395354997</t>
         </is>
       </c>
       <c r="R60" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370395354997</t>
         </is>
       </c>
     </row>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="N61" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O61" s="23" t="inlineStr">
@@ -6822,12 +6822,12 @@
       </c>
       <c r="Q61" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSC9946388102</t>
         </is>
       </c>
       <c r="R61" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSC9946388102</t>
         </is>
       </c>
     </row>
@@ -6895,7 +6895,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>SELF FULFILED</t>
         </is>
       </c>
       <c r="O62" s="19" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="K63" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Not Contactable</t>
         </is>
       </c>
       <c r="L63" s="24" t="inlineStr">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="N63" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>UNDELIVERED-3RD ATTEMPT</t>
         </is>
       </c>
       <c r="O63" s="23" t="inlineStr">
@@ -6998,12 +6998,12 @@
       </c>
       <c r="Q63" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3576445793KR</t>
         </is>
       </c>
       <c r="R63" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3576445793KR</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7071,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O64" s="19" t="inlineStr">
@@ -7086,12 +7086,12 @@
       </c>
       <c r="Q64" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSC3884345902</t>
         </is>
       </c>
       <c r="R64" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSC3884345902</t>
         </is>
       </c>
     </row>
@@ -7159,7 +7159,7 @@
       </c>
       <c r="N65" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O65" s="23" t="inlineStr">
@@ -7174,12 +7174,12 @@
       </c>
       <c r="Q65" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370384504495</t>
         </is>
       </c>
       <c r="R65" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370384504495</t>
         </is>
       </c>
     </row>
@@ -7247,7 +7247,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O66" s="19" t="inlineStr">
@@ -7262,12 +7262,12 @@
       </c>
       <c r="Q66" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSP2020476035</t>
         </is>
       </c>
       <c r="R66" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSP2020476035</t>
         </is>
       </c>
     </row>
@@ -7335,7 +7335,7 @@
       </c>
       <c r="N67" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>SELF FULFILED</t>
         </is>
       </c>
       <c r="O67" s="23" t="inlineStr">
@@ -7398,17 +7398,17 @@
       </c>
       <c r="I68" s="19" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J68" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K68" s="20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Refused To Accept   Otp Verified</t>
         </is>
       </c>
       <c r="L68" s="20" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="N68" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O68" s="19" t="inlineStr">
@@ -7438,12 +7438,12 @@
       </c>
       <c r="Q68" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1319460341769</t>
         </is>
       </c>
       <c r="R68" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/1319460341769</t>
         </is>
       </c>
     </row>
@@ -7486,17 +7486,17 @@
       </c>
       <c r="I69" s="23" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J69" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K69" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Refused To Accept   Otp Verified</t>
         </is>
       </c>
       <c r="L69" s="24" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="N69" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O69" s="23" t="inlineStr">
@@ -7526,12 +7526,12 @@
       </c>
       <c r="Q69" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1319460341773</t>
         </is>
       </c>
       <c r="R69" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/1319460341773</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="N70" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O70" s="19" t="inlineStr">
@@ -7614,12 +7614,12 @@
       </c>
       <c r="Q70" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112362553816</t>
         </is>
       </c>
       <c r="R70" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112362553816</t>
         </is>
       </c>
     </row>
@@ -7687,7 +7687,7 @@
       </c>
       <c r="N71" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O71" s="23" t="inlineStr">
@@ -7702,12 +7702,12 @@
       </c>
       <c r="Q71" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSP8409363746</t>
         </is>
       </c>
       <c r="R71" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSP8409363746</t>
         </is>
       </c>
     </row>
@@ -7775,7 +7775,7 @@
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O72" s="19" t="inlineStr">
@@ -7790,12 +7790,12 @@
       </c>
       <c r="Q72" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363889759</t>
         </is>
       </c>
       <c r="R72" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363889759</t>
         </is>
       </c>
     </row>
@@ -7857,14 +7857,14 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
     <col width="31" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="27" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -8023,7 +8023,7 @@
       </c>
       <c r="N2" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O2" s="19" t="inlineStr">
@@ -8038,12 +8038,12 @@
       </c>
       <c r="Q2" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112365216334</t>
         </is>
       </c>
       <c r="R2" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112365216334</t>
         </is>
       </c>
     </row>
@@ -8111,12 +8111,12 @@
       </c>
       <c r="N3" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O3" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P3" s="23" t="inlineStr">
@@ -8126,12 +8126,12 @@
       </c>
       <c r="Q3" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370503334064</t>
         </is>
       </c>
       <c r="R3" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370503334064</t>
         </is>
       </c>
     </row>
@@ -8199,7 +8199,7 @@
       </c>
       <c r="N4" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O4" s="19" t="inlineStr">
@@ -8214,12 +8214,12 @@
       </c>
       <c r="Q4" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370503560906</t>
         </is>
       </c>
       <c r="R4" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370503560906</t>
         </is>
       </c>
     </row>
@@ -8287,12 +8287,12 @@
       </c>
       <c r="N5" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O5" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P5" s="23" t="inlineStr">
@@ -8302,12 +8302,12 @@
       </c>
       <c r="Q5" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041932647740</t>
         </is>
       </c>
       <c r="R5" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041932647740</t>
         </is>
       </c>
     </row>
@@ -8375,12 +8375,12 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O6" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P6" s="19" t="inlineStr">
@@ -8390,12 +8390,12 @@
       </c>
       <c r="Q6" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370494726459</t>
         </is>
       </c>
       <c r="R6" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370494726459</t>
         </is>
       </c>
     </row>
@@ -8463,7 +8463,7 @@
       </c>
       <c r="N7" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O7" s="23" t="inlineStr">
@@ -8478,12 +8478,12 @@
       </c>
       <c r="Q7" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131169474</t>
         </is>
       </c>
       <c r="R7" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131169474</t>
         </is>
       </c>
     </row>
@@ -8551,7 +8551,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>UNDELIVERED-1ST ATTEMPT</t>
         </is>
       </c>
       <c r="O8" s="19" t="inlineStr">
@@ -8566,12 +8566,12 @@
       </c>
       <c r="Q8" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSC0319007800</t>
         </is>
       </c>
       <c r="R8" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSC0319007800</t>
         </is>
       </c>
     </row>
@@ -8614,17 +8614,17 @@
       </c>
       <c r="I9" s="23" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J9" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K9" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Cancelled Otp Verified</t>
         </is>
       </c>
       <c r="L9" s="24" t="inlineStr">
@@ -8639,7 +8639,7 @@
       </c>
       <c r="N9" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO IN TRANSIT</t>
         </is>
       </c>
       <c r="O9" s="23" t="inlineStr">
@@ -8654,12 +8654,12 @@
       </c>
       <c r="Q9" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3593208175KR</t>
         </is>
       </c>
       <c r="R9" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3593208175KR</t>
         </is>
       </c>
     </row>
@@ -8702,17 +8702,17 @@
       </c>
       <c r="I10" s="19" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J10" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Refused To Accept   Otp Verified</t>
         </is>
       </c>
       <c r="L10" s="20" t="inlineStr">
@@ -8727,7 +8727,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O10" s="19" t="inlineStr">
@@ -8742,12 +8742,12 @@
       </c>
       <c r="Q10" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112364415189</t>
         </is>
       </c>
       <c r="R10" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112364415189</t>
         </is>
       </c>
     </row>
@@ -8815,7 +8815,7 @@
       </c>
       <c r="N11" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O11" s="23" t="inlineStr">
@@ -8830,12 +8830,12 @@
       </c>
       <c r="Q11" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSC9436482183</t>
         </is>
       </c>
       <c r="R11" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSC9436482183</t>
         </is>
       </c>
     </row>
@@ -8903,7 +8903,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O12" s="19" t="inlineStr">
@@ -8918,12 +8918,12 @@
       </c>
       <c r="Q12" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3158678399SPF</t>
         </is>
       </c>
       <c r="R12" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3158678399SPF</t>
         </is>
       </c>
     </row>
@@ -8991,7 +8991,7 @@
       </c>
       <c r="N13" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O13" s="23" t="inlineStr">
@@ -9006,12 +9006,12 @@
       </c>
       <c r="Q13" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363521699</t>
         </is>
       </c>
       <c r="R13" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363521699</t>
         </is>
       </c>
     </row>
@@ -9079,7 +9079,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O14" s="19" t="inlineStr">
@@ -9094,12 +9094,12 @@
       </c>
       <c r="Q14" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112364314371</t>
         </is>
       </c>
       <c r="R14" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112364314371</t>
         </is>
       </c>
     </row>
@@ -9167,7 +9167,7 @@
       </c>
       <c r="N15" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O15" s="23" t="inlineStr">
@@ -9182,12 +9182,12 @@
       </c>
       <c r="Q15" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363687734</t>
         </is>
       </c>
       <c r="R15" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363687734</t>
         </is>
       </c>
     </row>
@@ -9255,7 +9255,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O16" s="19" t="inlineStr">
@@ -9270,12 +9270,12 @@
       </c>
       <c r="Q16" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370430051263</t>
         </is>
       </c>
       <c r="R16" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370430051263</t>
         </is>
       </c>
     </row>
@@ -9343,12 +9343,12 @@
       </c>
       <c r="N17" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O17" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P17" s="23" t="inlineStr">
@@ -9358,12 +9358,12 @@
       </c>
       <c r="Q17" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112367080297</t>
         </is>
       </c>
       <c r="R17" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112367080297</t>
         </is>
       </c>
     </row>
@@ -9431,7 +9431,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O18" s="19" t="inlineStr">
@@ -9446,12 +9446,12 @@
       </c>
       <c r="Q18" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370429882984</t>
         </is>
       </c>
       <c r="R18" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370429882984</t>
         </is>
       </c>
     </row>
@@ -9519,7 +9519,7 @@
       </c>
       <c r="N19" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O19" s="23" t="inlineStr">
@@ -9534,12 +9534,12 @@
       </c>
       <c r="Q19" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112365054938</t>
         </is>
       </c>
       <c r="R19" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112365054938</t>
         </is>
       </c>
     </row>
@@ -9607,12 +9607,12 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O20" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P20" s="19" t="inlineStr">
@@ -9622,12 +9622,12 @@
       </c>
       <c r="Q20" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3586915332KR</t>
         </is>
       </c>
       <c r="R20" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3586915332KR</t>
         </is>
       </c>
     </row>
@@ -9695,7 +9695,7 @@
       </c>
       <c r="N21" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O21" s="23" t="inlineStr">
@@ -9710,12 +9710,12 @@
       </c>
       <c r="Q21" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112362848987</t>
         </is>
       </c>
       <c r="R21" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112362848987</t>
         </is>
       </c>
     </row>
@@ -9768,7 +9768,7 @@
       </c>
       <c r="K22" s="20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customerunavailable Deliveryattempted</t>
         </is>
       </c>
       <c r="L22" s="20" t="inlineStr">
@@ -9783,7 +9783,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>UNDELIVERED-3RD ATTEMPT</t>
         </is>
       </c>
       <c r="O22" s="19" t="inlineStr">
@@ -9798,12 +9798,12 @@
       </c>
       <c r="Q22" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370429573110</t>
         </is>
       </c>
       <c r="R22" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370429573110</t>
         </is>
       </c>
     </row>
@@ -9846,17 +9846,17 @@
       </c>
       <c r="I23" s="23" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J23" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K23" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Not Available X Office Or Residence Closed</t>
         </is>
       </c>
       <c r="L23" s="24" t="inlineStr">
@@ -9871,7 +9871,7 @@
       </c>
       <c r="N23" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO IN TRANSIT</t>
         </is>
       </c>
       <c r="O23" s="23" t="inlineStr">
@@ -9886,12 +9886,12 @@
       </c>
       <c r="Q23" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363585911</t>
         </is>
       </c>
       <c r="R23" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363585911</t>
         </is>
       </c>
     </row>
@@ -9944,7 +9944,7 @@
       </c>
       <c r="K24" s="20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Receiver Requested Delivery On Another Date (Cir)</t>
         </is>
       </c>
       <c r="L24" s="20" t="inlineStr">
@@ -9959,7 +9959,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>UNDELIVERED-1ST ATTEMPT</t>
         </is>
       </c>
       <c r="O24" s="19" t="inlineStr">
@@ -9974,12 +9974,12 @@
       </c>
       <c r="Q24" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131457369</t>
         </is>
       </c>
       <c r="R24" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131457369</t>
         </is>
       </c>
     </row>
@@ -10047,7 +10047,7 @@
       </c>
       <c r="N25" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O25" s="23" t="inlineStr">
@@ -10062,12 +10062,12 @@
       </c>
       <c r="Q25" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370395354997</t>
         </is>
       </c>
       <c r="R25" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370395354997</t>
         </is>
       </c>
     </row>
@@ -10135,7 +10135,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O26" s="19" t="inlineStr">
@@ -10150,12 +10150,12 @@
       </c>
       <c r="Q26" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSC9946388102</t>
         </is>
       </c>
       <c r="R26" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSC9946388102</t>
         </is>
       </c>
     </row>
@@ -10223,7 +10223,7 @@
       </c>
       <c r="N27" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>SELF FULFILED</t>
         </is>
       </c>
       <c r="O27" s="23" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="K28" s="20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Not Contactable</t>
         </is>
       </c>
       <c r="L28" s="20" t="inlineStr">
@@ -10311,7 +10311,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>UNDELIVERED-3RD ATTEMPT</t>
         </is>
       </c>
       <c r="O28" s="19" t="inlineStr">
@@ -10326,12 +10326,12 @@
       </c>
       <c r="Q28" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3576445793KR</t>
         </is>
       </c>
       <c r="R28" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3576445793KR</t>
         </is>
       </c>
     </row>
@@ -10399,7 +10399,7 @@
       </c>
       <c r="N29" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O29" s="23" t="inlineStr">
@@ -10414,12 +10414,12 @@
       </c>
       <c r="Q29" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSC3884345902</t>
         </is>
       </c>
       <c r="R29" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSC3884345902</t>
         </is>
       </c>
     </row>
@@ -10487,7 +10487,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O30" s="19" t="inlineStr">
@@ -10502,12 +10502,12 @@
       </c>
       <c r="Q30" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370384504495</t>
         </is>
       </c>
       <c r="R30" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370384504495</t>
         </is>
       </c>
     </row>
@@ -10575,7 +10575,7 @@
       </c>
       <c r="N31" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O31" s="23" t="inlineStr">
@@ -10590,12 +10590,12 @@
       </c>
       <c r="Q31" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSP2020476035</t>
         </is>
       </c>
       <c r="R31" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSP2020476035</t>
         </is>
       </c>
     </row>
@@ -10663,7 +10663,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>SELF FULFILED</t>
         </is>
       </c>
       <c r="O32" s="19" t="inlineStr">
@@ -10726,17 +10726,17 @@
       </c>
       <c r="I33" s="23" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K33" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Refused To Accept   Otp Verified</t>
         </is>
       </c>
       <c r="L33" s="24" t="inlineStr">
@@ -10751,7 +10751,7 @@
       </c>
       <c r="N33" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O33" s="23" t="inlineStr">
@@ -10766,12 +10766,12 @@
       </c>
       <c r="Q33" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1319460341769</t>
         </is>
       </c>
       <c r="R33" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/1319460341769</t>
         </is>
       </c>
     </row>
@@ -10814,17 +10814,17 @@
       </c>
       <c r="I34" s="19" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J34" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K34" s="20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Refused To Accept   Otp Verified</t>
         </is>
       </c>
       <c r="L34" s="20" t="inlineStr">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO OFD</t>
         </is>
       </c>
       <c r="O34" s="19" t="inlineStr">
@@ -10854,12 +10854,12 @@
       </c>
       <c r="Q34" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1319460341773</t>
         </is>
       </c>
       <c r="R34" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/1319460341773</t>
         </is>
       </c>
     </row>
@@ -10927,7 +10927,7 @@
       </c>
       <c r="N35" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O35" s="23" t="inlineStr">
@@ -10942,12 +10942,12 @@
       </c>
       <c r="Q35" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112362553816</t>
         </is>
       </c>
       <c r="R35" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112362553816</t>
         </is>
       </c>
     </row>
@@ -11015,7 +11015,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O36" s="19" t="inlineStr">
@@ -11030,12 +11030,12 @@
       </c>
       <c r="Q36" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSP8409363746</t>
         </is>
       </c>
       <c r="R36" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSP8409363746</t>
         </is>
       </c>
     </row>
@@ -11103,7 +11103,7 @@
       </c>
       <c r="N37" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O37" s="23" t="inlineStr">
@@ -11118,12 +11118,12 @@
       </c>
       <c r="Q37" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363889759</t>
         </is>
       </c>
       <c r="R37" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363889759</t>
         </is>
       </c>
     </row>
@@ -11185,14 +11185,14 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="33" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -11703,7 +11703,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O6" s="19" t="inlineStr">
@@ -11791,7 +11791,7 @@
       </c>
       <c r="N7" s="23" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O7" s="23" t="inlineStr">
@@ -11879,7 +11879,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>NEW ORDER</t>
         </is>
       </c>
       <c r="O8" s="19" t="inlineStr">
@@ -11967,7 +11967,7 @@
       </c>
       <c r="N9" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O9" s="23" t="inlineStr">
@@ -11982,12 +11982,12 @@
       </c>
       <c r="Q9" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3158681570SPF</t>
         </is>
       </c>
       <c r="R9" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3158681570SPF</t>
         </is>
       </c>
     </row>
@@ -12055,7 +12055,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O10" s="19" t="inlineStr">
@@ -12070,12 +12070,12 @@
       </c>
       <c r="Q10" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041933834995</t>
         </is>
       </c>
       <c r="R10" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041933834995</t>
         </is>
       </c>
     </row>
@@ -12143,7 +12143,7 @@
       </c>
       <c r="N11" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O11" s="23" t="inlineStr">
@@ -12158,12 +12158,12 @@
       </c>
       <c r="Q11" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041933767110</t>
         </is>
       </c>
       <c r="R11" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041933767110</t>
         </is>
       </c>
     </row>
@@ -12231,7 +12231,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O12" s="19" t="inlineStr">
@@ -12246,12 +12246,12 @@
       </c>
       <c r="Q12" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3158681535SPF</t>
         </is>
       </c>
       <c r="R12" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3158681535SPF</t>
         </is>
       </c>
     </row>
@@ -12319,7 +12319,7 @@
       </c>
       <c r="N13" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>OUT FOR PICKUP</t>
         </is>
       </c>
       <c r="O13" s="23" t="inlineStr">
@@ -12334,12 +12334,12 @@
       </c>
       <c r="Q13" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D125041276</t>
         </is>
       </c>
       <c r="R13" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D125041276</t>
         </is>
       </c>
     </row>
@@ -12407,7 +12407,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>IN TRANSIT-EN-ROUTE</t>
         </is>
       </c>
       <c r="O14" s="19" t="inlineStr">
@@ -12422,12 +12422,12 @@
       </c>
       <c r="Q14" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>143263608413636</t>
         </is>
       </c>
       <c r="R14" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/143263608413636</t>
         </is>
       </c>
     </row>
@@ -12495,7 +12495,7 @@
       </c>
       <c r="N15" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP SCHEDULED</t>
         </is>
       </c>
       <c r="O15" s="23" t="inlineStr">
@@ -12510,12 +12510,12 @@
       </c>
       <c r="Q15" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3622719795KR</t>
         </is>
       </c>
       <c r="R15" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3622719795KR</t>
         </is>
       </c>
     </row>
@@ -12583,7 +12583,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O16" s="19" t="inlineStr">
@@ -12598,12 +12598,12 @@
       </c>
       <c r="Q16" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041933357982</t>
         </is>
       </c>
       <c r="R16" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041933357982</t>
         </is>
       </c>
     </row>
@@ -12671,7 +12671,7 @@
       </c>
       <c r="N17" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>IN TRANSIT-AT DESTINATION HUB</t>
         </is>
       </c>
       <c r="O17" s="23" t="inlineStr">
@@ -12686,12 +12686,12 @@
       </c>
       <c r="Q17" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041933358111</t>
         </is>
       </c>
       <c r="R17" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041933358111</t>
         </is>
       </c>
     </row>
@@ -12759,7 +12759,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>IN TRANSIT-EN-ROUTE</t>
         </is>
       </c>
       <c r="O18" s="19" t="inlineStr">
@@ -12774,12 +12774,12 @@
       </c>
       <c r="Q18" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19041933375224</t>
         </is>
       </c>
       <c r="R18" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/19041933375224</t>
         </is>
       </c>
     </row>
@@ -12847,7 +12847,7 @@
       </c>
       <c r="N19" s="23" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O19" s="23" t="inlineStr">
@@ -12862,12 +12862,12 @@
       </c>
       <c r="Q19" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>143263612093343</t>
         </is>
       </c>
       <c r="R19" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/143263612093343</t>
         </is>
       </c>
     </row>
@@ -12935,7 +12935,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>IN TRANSIT</t>
         </is>
       </c>
       <c r="O20" s="19" t="inlineStr">
@@ -12950,12 +12950,12 @@
       </c>
       <c r="Q20" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370577344761</t>
         </is>
       </c>
       <c r="R20" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370577344761</t>
         </is>
       </c>
     </row>
@@ -13023,7 +13023,7 @@
       </c>
       <c r="N21" s="23" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>IN TRANSIT-EN-ROUTE</t>
         </is>
       </c>
       <c r="O21" s="23" t="inlineStr">
@@ -13038,12 +13038,12 @@
       </c>
       <c r="Q21" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112362996290</t>
         </is>
       </c>
       <c r="R21" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112362996290</t>
         </is>
       </c>
     </row>
@@ -13111,7 +13111,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O22" s="19" t="inlineStr">
@@ -13126,12 +13126,12 @@
       </c>
       <c r="Q22" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>143263608436527</t>
         </is>
       </c>
       <c r="R22" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/143263608436527</t>
         </is>
       </c>
     </row>
@@ -13199,7 +13199,7 @@
       </c>
       <c r="N23" s="23" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O23" s="23" t="inlineStr">
@@ -13214,12 +13214,12 @@
       </c>
       <c r="Q23" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370574614355</t>
         </is>
       </c>
       <c r="R23" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370574614355</t>
         </is>
       </c>
     </row>
@@ -13287,12 +13287,12 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O24" s="19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P24" s="19" t="inlineStr">
@@ -13302,12 +13302,12 @@
       </c>
       <c r="Q24" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3158680701SPF</t>
         </is>
       </c>
       <c r="R24" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3158680701SPF</t>
         </is>
       </c>
     </row>
@@ -13375,7 +13375,7 @@
       </c>
       <c r="N25" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>OUT FOR DELIVERY</t>
         </is>
       </c>
       <c r="O25" s="23" t="inlineStr">
@@ -13390,12 +13390,12 @@
       </c>
       <c r="Q25" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370554649599</t>
         </is>
       </c>
       <c r="R25" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370554649599</t>
         </is>
       </c>
     </row>
@@ -13463,7 +13463,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>DELIVERED</t>
         </is>
       </c>
       <c r="O26" s="19" t="inlineStr">
@@ -13478,12 +13478,12 @@
       </c>
       <c r="Q26" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370552365989</t>
         </is>
       </c>
       <c r="R26" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370552365989</t>
         </is>
       </c>
     </row>
@@ -13536,7 +13536,7 @@
       </c>
       <c r="K27" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pickup Not Attempted</t>
         </is>
       </c>
       <c r="L27" s="24" t="inlineStr">
@@ -13551,7 +13551,7 @@
       </c>
       <c r="N27" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O27" s="23" t="inlineStr">
@@ -13566,12 +13566,12 @@
       </c>
       <c r="Q27" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1091393193440</t>
         </is>
       </c>
       <c r="R27" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/1091393193440</t>
         </is>
       </c>
     </row>
@@ -13639,7 +13639,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O28" s="19" t="inlineStr">
@@ -13654,12 +13654,12 @@
       </c>
       <c r="Q28" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3158680814SPF</t>
         </is>
       </c>
       <c r="R28" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3158680814SPF</t>
         </is>
       </c>
     </row>
@@ -13727,7 +13727,7 @@
       </c>
       <c r="N29" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP EXCEPTION</t>
         </is>
       </c>
       <c r="O29" s="23" t="inlineStr">
@@ -13742,12 +13742,12 @@
       </c>
       <c r="Q29" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131505337</t>
         </is>
       </c>
       <c r="R29" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131505337</t>
         </is>
       </c>
     </row>
@@ -13815,7 +13815,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>IN TRANSIT</t>
         </is>
       </c>
       <c r="O30" s="19" t="inlineStr">
@@ -13830,12 +13830,12 @@
       </c>
       <c r="Q30" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370553698802</t>
         </is>
       </c>
       <c r="R30" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370553698802</t>
         </is>
       </c>
     </row>
@@ -13903,7 +13903,7 @@
       </c>
       <c r="N31" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>REACHED DESTINATION HUB</t>
         </is>
       </c>
       <c r="O31" s="23" t="inlineStr">
@@ -13918,12 +13918,12 @@
       </c>
       <c r="Q31" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370550963576</t>
         </is>
       </c>
       <c r="R31" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370550963576</t>
         </is>
       </c>
     </row>
@@ -13991,7 +13991,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>CANCELED</t>
         </is>
       </c>
       <c r="O32" s="19" t="inlineStr">
@@ -14006,12 +14006,12 @@
       </c>
       <c r="Q32" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112362403829</t>
         </is>
       </c>
       <c r="R32" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112362403829</t>
         </is>
       </c>
     </row>
@@ -14064,7 +14064,7 @@
       </c>
       <c r="K33" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pickup Not Attempted</t>
         </is>
       </c>
       <c r="L33" s="24" t="inlineStr">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="N33" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>OUT FOR DELIVERY</t>
         </is>
       </c>
       <c r="O33" s="23" t="inlineStr">
@@ -14094,12 +14094,12 @@
       </c>
       <c r="Q33" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1091393138630</t>
         </is>
       </c>
       <c r="R33" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/1091393138630</t>
         </is>
       </c>
     </row>
@@ -14167,7 +14167,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP EXCEPTION</t>
         </is>
       </c>
       <c r="O34" s="19" t="inlineStr">
@@ -14182,12 +14182,12 @@
       </c>
       <c r="Q34" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131502192</t>
         </is>
       </c>
       <c r="R34" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131502192</t>
         </is>
       </c>
     </row>
@@ -14255,7 +14255,7 @@
       </c>
       <c r="N35" s="23" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>PICKUP EXCEPTION</t>
         </is>
       </c>
       <c r="O35" s="23" t="inlineStr">
@@ -14270,12 +14270,12 @@
       </c>
       <c r="Q35" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131501705</t>
         </is>
       </c>
       <c r="R35" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131501705</t>
         </is>
       </c>
     </row>
@@ -14328,7 +14328,7 @@
       </c>
       <c r="K36" s="20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Deliveryattempted Unabletocontactrecipient</t>
         </is>
       </c>
       <c r="L36" s="20" t="inlineStr">
@@ -14343,7 +14343,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>UNDELIVERED</t>
         </is>
       </c>
       <c r="O36" s="19" t="inlineStr">
@@ -14358,12 +14358,12 @@
       </c>
       <c r="Q36" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370526573181</t>
         </is>
       </c>
       <c r="R36" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370526573181</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split camelCase and PascalCase Shiprocket reason comments with spaces
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -4592,7 +4592,7 @@
       </c>
       <c r="K36" s="20" t="inlineStr">
         <is>
-          <t>Deliveryattempted Unabletocontactrecipient</t>
+          <t>Delivery Attempted Unable To Contact Recipient</t>
         </is>
       </c>
       <c r="L36" s="20" t="inlineStr">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="K44" s="20" t="inlineStr">
         <is>
-          <t>Customer Cancelled Otp Verified</t>
+          <t>Customer Cancelled O T P Verified</t>
         </is>
       </c>
       <c r="L44" s="20" t="inlineStr">
@@ -5384,7 +5384,7 @@
       </c>
       <c r="K45" s="24" t="inlineStr">
         <is>
-          <t>Customer Refused To Accept   Otp Verified</t>
+          <t>Customer Refused To Accept O T P Verified</t>
         </is>
       </c>
       <c r="L45" s="24" t="inlineStr">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="K57" s="24" t="inlineStr">
         <is>
-          <t>Customerunavailable Deliveryattempted</t>
+          <t>Customer Unavailable Delivery Attempted</t>
         </is>
       </c>
       <c r="L57" s="24" t="inlineStr">
@@ -7408,7 +7408,7 @@
       </c>
       <c r="K68" s="20" t="inlineStr">
         <is>
-          <t>Customer Refused To Accept   Otp Verified</t>
+          <t>Customer Refused To Accept O T P Verified</t>
         </is>
       </c>
       <c r="L68" s="20" t="inlineStr">
@@ -7496,7 +7496,7 @@
       </c>
       <c r="K69" s="24" t="inlineStr">
         <is>
-          <t>Customer Refused To Accept   Otp Verified</t>
+          <t>Customer Refused To Accept O T P Verified</t>
         </is>
       </c>
       <c r="L69" s="24" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="K9" s="24" t="inlineStr">
         <is>
-          <t>Customer Cancelled Otp Verified</t>
+          <t>Customer Cancelled O T P Verified</t>
         </is>
       </c>
       <c r="L9" s="24" t="inlineStr">
@@ -8712,7 +8712,7 @@
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>Customer Refused To Accept   Otp Verified</t>
+          <t>Customer Refused To Accept O T P Verified</t>
         </is>
       </c>
       <c r="L10" s="20" t="inlineStr">
@@ -9768,7 +9768,7 @@
       </c>
       <c r="K22" s="20" t="inlineStr">
         <is>
-          <t>Customerunavailable Deliveryattempted</t>
+          <t>Customer Unavailable Delivery Attempted</t>
         </is>
       </c>
       <c r="L22" s="20" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="K33" s="24" t="inlineStr">
         <is>
-          <t>Customer Refused To Accept   Otp Verified</t>
+          <t>Customer Refused To Accept O T P Verified</t>
         </is>
       </c>
       <c r="L33" s="24" t="inlineStr">
@@ -10824,7 +10824,7 @@
       </c>
       <c r="K34" s="20" t="inlineStr">
         <is>
-          <t>Customer Refused To Accept   Otp Verified</t>
+          <t>Customer Refused To Accept O T P Verified</t>
         </is>
       </c>
       <c r="L34" s="20" t="inlineStr">
@@ -11185,7 +11185,7 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="46" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="33" customWidth="1" min="14" max="14"/>
@@ -14328,7 +14328,7 @@
       </c>
       <c r="K36" s="20" t="inlineStr">
         <is>
-          <t>Deliveryattempted Unabletocontactrecipient</t>
+          <t>Delivery Attempted Unable To Contact Recipient</t>
         </is>
       </c>
       <c r="L36" s="20" t="inlineStr">

</xml_diff>

<commit_message>
Align returned count: exclude Delivered/Self Fulfilled from returned in KPI cards and Excel
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -718,10 +718,10 @@
         <v>188590</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>20662</v>
+        <v>17486</v>
       </c>
       <c r="F4" s="6" t="n">
         <v>6</v>
@@ -769,10 +769,10 @@
         <v>81</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>149506</v>
+        <v>152682</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.1228070175438596</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="F7" s="11" t="n">
         <v>0.3333333333333333</v>

</xml_diff>

<commit_message>
feat: Add custom dual-pane date range picker, CO-ORD SET category, dynamic 12-column category grid, and logistics pipeline updates
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -3892,7 +3892,7 @@
       </c>
       <c r="P22" s="22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q22" s="22" t="inlineStr">
@@ -21782,7 +21782,7 @@
       </c>
       <c r="P22" s="22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q22" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Fix deniedList filter in app.js and generate_sheet.py to exclude DELIVERED orders so count equals strictly 15
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -847,12 +847,12 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>16 (₹25,622.00)</t>
+          <t>15 (₹23,478.00)</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>4 (₹6,280.00)</t>
+          <t>5 (₹8,424.00)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Include REACHED BACK AT_SELLER_CITY status in RTO filter pattern so Denied Orders count equals 15
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -757,11 +757,11 @@
         <v>391979</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>340033</v>
+        <v>336463</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>~ ₹2,394.60</t>
+          <t>~ ₹2,369.46</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>14 (₹19,908.00)</t>
+          <t>15 (₹23,478.00)</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Add clean Category Summary tab and sync to Google Sheets
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Jan 2027" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Feb 2027" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Mar 2027" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Category Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,12 +28,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
     <numFmt numFmtId="166" formatCode="dd-mm-yyyy"/>
     <numFmt numFmtId="167" formatCode="₹#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="mmm yyyy"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="mmm yyyy"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -225,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -286,7 +288,7 @@
     <xf numFmtId="167" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -298,7 +300,7 @@
     <xf numFmtId="167" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -334,6 +336,30 @@
     </xf>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2384,6 +2410,343 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Total Orders</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>Delivered Orders</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Share (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>TOPS</t>
+        </is>
+      </c>
+      <c r="B2" s="39" t="n">
+        <v>216</v>
+      </c>
+      <c r="C2" s="40" t="n">
+        <v>390201.34</v>
+      </c>
+      <c r="D2" s="39" t="n">
+        <v>195</v>
+      </c>
+      <c r="E2" s="41" t="n">
+        <v>0.5490653264340458</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="31" t="inlineStr">
+        <is>
+          <t>CHUDIDHAR</t>
+        </is>
+      </c>
+      <c r="B3" s="42" t="n">
+        <v>67</v>
+      </c>
+      <c r="C3" s="43" t="n">
+        <v>159679.35</v>
+      </c>
+      <c r="D3" s="42" t="n">
+        <v>49</v>
+      </c>
+      <c r="E3" s="44" t="n">
+        <v>0.2246901418445315</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>ANARKALI</t>
+        </is>
+      </c>
+      <c r="B4" s="39" t="n">
+        <v>39</v>
+      </c>
+      <c r="C4" s="40" t="n">
+        <v>168321</v>
+      </c>
+      <c r="D4" s="39" t="n">
+        <v>35</v>
+      </c>
+      <c r="E4" s="41" t="n">
+        <v>0.2368500959292068</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>LEHENGA</t>
+        </is>
+      </c>
+      <c r="B5" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="43" t="n">
+        <v>13829</v>
+      </c>
+      <c r="D5" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="44" t="n">
+        <v>0.01945924737023307</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>CO-ORD SET</t>
+        </is>
+      </c>
+      <c r="B6" s="39" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" s="40" t="n">
+        <v>22490</v>
+      </c>
+      <c r="D6" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" s="41" t="n">
+        <v>0.03164642948561297</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>HALF SAREE LEHENGA</t>
+        </is>
+      </c>
+      <c r="B7" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="43" t="n">
+        <v>2950</v>
+      </c>
+      <c r="D7" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="44" t="n">
+        <v>0.004151043440754036</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>LONG GOWN</t>
+        </is>
+      </c>
+      <c r="B8" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="40" t="n">
+        <v>11182</v>
+      </c>
+      <c r="D8" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="41" t="n">
+        <v>0.01573456534051242</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="31" t="inlineStr">
+        <is>
+          <t>SHARARA</t>
+        </is>
+      </c>
+      <c r="B9" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="43" t="n">
+        <v>1940</v>
+      </c>
+      <c r="D9" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="44" t="n">
+        <v>0.002729838737309434</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>DRESS</t>
+        </is>
+      </c>
+      <c r="B10" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>KURTI</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>SAREE</t>
+        </is>
+      </c>
+      <c r="B12" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="40" t="n">
+        <v>2950</v>
+      </c>
+      <c r="D12" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="41" t="n">
+        <v>0.004151043440754036</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="C13" s="43" t="n">
+        <v>22490</v>
+      </c>
+      <c r="D13" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" s="44" t="n">
+        <v>0.03164642948561297</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>SUIT</t>
+        </is>
+      </c>
+      <c r="B14" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="31" t="inlineStr">
+        <is>
+          <t>OTHERS</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="C15" s="43" t="n">
+        <v>22490</v>
+      </c>
+      <c r="D15" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="44" t="n">
+        <v>0.03164642948561297</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="36" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B16" s="45">
+        <f>SUM(B2:B15)</f>
+        <v/>
+      </c>
+      <c r="C16" s="38">
+        <f>SUM(C2:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="45">
+        <f>SUM(D2:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="46">
+        <f>SUM(E2:E15)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Remove Category Summary tab completely from local Excel and Google Sheets
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -19,7 +19,6 @@
     <sheet name="Jan 2027" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Feb 2027" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Mar 2027" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Category Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,13 +27,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
     <numFmt numFmtId="166" formatCode="dd-mm-yyyy"/>
     <numFmt numFmtId="167" formatCode="₹#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
-    <numFmt numFmtId="169" formatCode="mmm yyyy"/>
+    <numFmt numFmtId="168" formatCode="mmm yyyy"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -227,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -288,7 +286,7 @@
     <xf numFmtId="167" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -300,7 +298,7 @@
     <xf numFmtId="167" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -336,30 +334,6 @@
     </xf>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2410,343 +2384,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B1" s="18" t="inlineStr">
-        <is>
-          <t>Total Orders</t>
-        </is>
-      </c>
-      <c r="C1" s="18" t="inlineStr">
-        <is>
-          <t>Total Revenue</t>
-        </is>
-      </c>
-      <c r="D1" s="18" t="inlineStr">
-        <is>
-          <t>Delivered Orders</t>
-        </is>
-      </c>
-      <c r="E1" s="18" t="inlineStr">
-        <is>
-          <t>Revenue Share (%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>TOPS</t>
-        </is>
-      </c>
-      <c r="B2" s="39" t="n">
-        <v>216</v>
-      </c>
-      <c r="C2" s="40" t="n">
-        <v>390201.34</v>
-      </c>
-      <c r="D2" s="39" t="n">
-        <v>195</v>
-      </c>
-      <c r="E2" s="41" t="n">
-        <v>0.5490653264340458</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="31" t="inlineStr">
-        <is>
-          <t>CHUDIDHAR</t>
-        </is>
-      </c>
-      <c r="B3" s="42" t="n">
-        <v>67</v>
-      </c>
-      <c r="C3" s="43" t="n">
-        <v>159679.35</v>
-      </c>
-      <c r="D3" s="42" t="n">
-        <v>49</v>
-      </c>
-      <c r="E3" s="44" t="n">
-        <v>0.2246901418445315</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
-        <is>
-          <t>ANARKALI</t>
-        </is>
-      </c>
-      <c r="B4" s="39" t="n">
-        <v>39</v>
-      </c>
-      <c r="C4" s="40" t="n">
-        <v>168321</v>
-      </c>
-      <c r="D4" s="39" t="n">
-        <v>35</v>
-      </c>
-      <c r="E4" s="41" t="n">
-        <v>0.2368500959292068</v>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="31" t="inlineStr">
-        <is>
-          <t>LEHENGA</t>
-        </is>
-      </c>
-      <c r="B5" s="42" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" s="43" t="n">
-        <v>13829</v>
-      </c>
-      <c r="D5" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="44" t="n">
-        <v>0.01945924737023307</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
-        <is>
-          <t>CO-ORD SET</t>
-        </is>
-      </c>
-      <c r="B6" s="39" t="n">
-        <v>15</v>
-      </c>
-      <c r="C6" s="40" t="n">
-        <v>22490</v>
-      </c>
-      <c r="D6" s="39" t="n">
-        <v>8</v>
-      </c>
-      <c r="E6" s="41" t="n">
-        <v>0.03164642948561297</v>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="31" t="inlineStr">
-        <is>
-          <t>HALF SAREE LEHENGA</t>
-        </is>
-      </c>
-      <c r="B7" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="43" t="n">
-        <v>2950</v>
-      </c>
-      <c r="D7" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="44" t="n">
-        <v>0.004151043440754036</v>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>LONG GOWN</t>
-        </is>
-      </c>
-      <c r="B8" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="40" t="n">
-        <v>11182</v>
-      </c>
-      <c r="D8" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="41" t="n">
-        <v>0.01573456534051242</v>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="31" t="inlineStr">
-        <is>
-          <t>SHARARA</t>
-        </is>
-      </c>
-      <c r="B9" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="43" t="n">
-        <v>1940</v>
-      </c>
-      <c r="D9" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="44" t="n">
-        <v>0.002729838737309434</v>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="27" t="inlineStr">
-        <is>
-          <t>DRESS</t>
-        </is>
-      </c>
-      <c r="B10" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="41" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="31" t="inlineStr">
-        <is>
-          <t>KURTI</t>
-        </is>
-      </c>
-      <c r="B11" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="43" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="44" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="27" t="inlineStr">
-        <is>
-          <t>SAREE</t>
-        </is>
-      </c>
-      <c r="B12" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="40" t="n">
-        <v>2950</v>
-      </c>
-      <c r="D12" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="41" t="n">
-        <v>0.004151043440754036</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="31" t="inlineStr">
-        <is>
-          <t>SET</t>
-        </is>
-      </c>
-      <c r="B13" s="42" t="n">
-        <v>15</v>
-      </c>
-      <c r="C13" s="43" t="n">
-        <v>22490</v>
-      </c>
-      <c r="D13" s="42" t="n">
-        <v>8</v>
-      </c>
-      <c r="E13" s="44" t="n">
-        <v>0.03164642948561297</v>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="27" t="inlineStr">
-        <is>
-          <t>SUIT</t>
-        </is>
-      </c>
-      <c r="B14" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="41" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="31" t="inlineStr">
-        <is>
-          <t>OTHERS</t>
-        </is>
-      </c>
-      <c r="B15" s="42" t="n">
-        <v>15</v>
-      </c>
-      <c r="C15" s="43" t="n">
-        <v>22490</v>
-      </c>
-      <c r="D15" s="42" t="n">
-        <v>8</v>
-      </c>
-      <c r="E15" s="44" t="n">
-        <v>0.03164642948561297</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="36" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B16" s="45">
-        <f>SUM(B2:B15)</f>
-        <v/>
-      </c>
-      <c r="C16" s="38">
-        <f>SUM(C2:C15)</f>
-        <v/>
-      </c>
-      <c r="D16" s="45">
-        <f>SUM(D2:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="46">
-        <f>SUM(E2:E15)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>